<commit_message>
Atualiza dados das planilhas
</commit_message>
<xml_diff>
--- a/doc/EAP_PRODUCAO.xlsx
+++ b/doc/EAP_PRODUCAO.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\github_corrigido_dashboard_obrasRev1\github\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2299176A-C19C-40BD-A1D5-6456718FD83A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72C358BF-8DF4-4D62-BADE-D5393D7E8BF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EAP_PRODUCAO" sheetId="2" r:id="rId1"/>
@@ -953,7 +953,7 @@
         <v>2426.84</v>
       </c>
       <c r="E16" s="2">
-        <v>1747.73</v>
+        <v>1538.59</v>
       </c>
       <c r="F16">
         <v>2735</v>
@@ -963,7 +963,7 @@
       </c>
       <c r="I16" s="5">
         <f t="shared" si="0"/>
-        <v>679.11000000000013</v>
+        <v>888.25000000000023</v>
       </c>
       <c r="J16" s="5"/>
     </row>
@@ -1109,19 +1109,19 @@
     <row r="27" spans="2:16" x14ac:dyDescent="0.3">
       <c r="P27">
         <f>SUM(E3:E16)</f>
-        <v>15619.635000000002</v>
+        <v>15410.495000000003</v>
       </c>
     </row>
     <row r="28" spans="2:16" x14ac:dyDescent="0.3">
       <c r="P28">
         <f>14468.56-P27</f>
-        <v>-1151.0750000000025</v>
+        <v>-941.93500000000313</v>
       </c>
     </row>
     <row r="29" spans="2:16" x14ac:dyDescent="0.3">
       <c r="P29">
         <f>P28+2135.09</f>
-        <v>984.0149999999976</v>
+        <v>1193.154999999997</v>
       </c>
     </row>
     <row r="34" spans="8:8" x14ac:dyDescent="0.3">

</xml_diff>